<commit_message>
Release v0.6.1: group_random split mode and group leakage audit.
Add entity-level Train/Test split (PFM_BIZ_ID+INST_ID), 04 group audit, pipeline UI, and handoff for paused 05-10 run.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/outputs/reports/comparison/leakage_audit.xlsx
+++ b/outputs/reports/comparison/leakage_audit.xlsx
@@ -12,7 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="단변량(univariate)" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="의심피처(suspects)" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="라벨정의검증(label_def)" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="피처목록(feature_list)" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="그룹중복(group_overlap)" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="피처목록(feature_list)" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -418,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,7 +453,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.003245465363672425</v>
+        <v>0.003298540954145681</v>
       </c>
     </row>
     <row r="4">
@@ -494,6 +495,40 @@
       <c r="B7" t="inlineStr">
         <is>
           <t>단변량 ROC-AUC가 0.9 이상이면 타겟과 거의 같이 움직이는 피처일 수 있음. 다만 여러 피처가 중정도(0.7~0.85)만으로도 앙상블 AUC 0.97대는 충분히 가능.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>그룹중복판정(group_verdict)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>PASS_그룹중복_낮음</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>최대_이미양성으로본비율(group_worst_ratio)</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>그룹중복_해석가이드</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Test 양성 엔티티 중 Train에서 이미 양성으로 등장한 비율이 높으면, 지표가 '신규 대상 탐지'가 아니라 '기존 대상 재탐지' 성능을 재고 있을 수 있음. 랜덤분할기대중복비율과 비슷하면 원인은 행 단위 random 분할. 시간 분할(split.mode=time, 기간 겹침 금지) 또는 사업 단위 그룹 분할로 대조 권장.</t>
         </is>
       </c>
     </row>
@@ -615,17 +650,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AID_BZR_FNDN_YS</t>
+          <t>MBR_NUM</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.5953456177723242</v>
+        <v>0.6102765417449965</v>
       </c>
       <c r="C2" t="n">
-        <v>0.004388227477903696</v>
+        <v>0.005028550594959024</v>
       </c>
       <c r="D2" t="n">
-        <v>1.352110402108304</v>
+        <v>1.524477235499843</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -634,17 +669,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MBR_NUM</t>
+          <t>AID_BZR_FNDN_YS</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.5865129899625758</v>
+        <v>0.5998644155237193</v>
       </c>
       <c r="C3" t="n">
-        <v>0.00451154947971646</v>
+        <v>0.00454795316016301</v>
       </c>
       <c r="D3" t="n">
-        <v>1.390108651355746</v>
+        <v>1.378777230110495</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -653,17 +688,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>RPRSV_DSCRD_YN</t>
+          <t>BIZ_ENFC_ZON_DV_CD</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.5665283492279621</v>
+        <v>0.5761693939467283</v>
       </c>
       <c r="C4" t="n">
-        <v>0.003816934440223919</v>
+        <v>0.003972629328477104</v>
       </c>
       <c r="D4" t="n">
-        <v>1.176082321798328</v>
+        <v>1.204359558878362</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -672,17 +707,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>FTEP_STF_NUM</t>
+          <t>RPRSV_DSCRD_YN</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.5639898417659797</v>
+        <v>0.5711620781593952</v>
       </c>
       <c r="C5" t="n">
-        <v>0.004020446872672561</v>
+        <v>0.003930160815310115</v>
       </c>
       <c r="D5" t="n">
-        <v>1.238789024734253</v>
+        <v>1.19148462000164</v>
       </c>
       <c r="E5" t="b">
         <v>0</v>
@@ -691,17 +726,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BIZ_ENFC_ZON_DV_CD</t>
+          <t>FTEP_STF_NUM</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.5635780338585543</v>
+        <v>0.5615620562385282</v>
       </c>
       <c r="C6" t="n">
-        <v>0.003781455584011756</v>
+        <v>0.003990484660004932</v>
       </c>
       <c r="D6" t="n">
-        <v>1.165150497780333</v>
+        <v>1.209772658723427</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -710,17 +745,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BIZCT_PYHWY_AMT</t>
+          <t>OPCT_YN</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.5598697291247227</v>
+        <v>0.5586010024042695</v>
       </c>
       <c r="C7" t="n">
-        <v>0.003659745890894433</v>
+        <v>0.003873567996462748</v>
       </c>
       <c r="D7" t="n">
-        <v>1.127649036671039</v>
+        <v>1.174327695278229</v>
       </c>
       <c r="E7" t="b">
         <v>0</v>
@@ -729,17 +764,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>RPRSV_AGGP_DV_CD</t>
+          <t>BIZCT_PYHWY_AMT</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.55683852371723</v>
+        <v>0.551091824190286</v>
       </c>
       <c r="C8" t="n">
-        <v>0.005400036456637725</v>
+        <v>0.003688696469464779</v>
       </c>
       <c r="D8" t="n">
-        <v>1.663871233100231</v>
+        <v>1.118281240324981</v>
       </c>
       <c r="E8" t="b">
         <v>0</v>
@@ -748,17 +783,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CUMU_PYHWY_EXE_CNT</t>
+          <t>RPRSV_AGGP_DV_CD</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.5476144328059797</v>
+        <v>0.5504587929986074</v>
       </c>
       <c r="C9" t="n">
-        <v>0.003792557774419537</v>
+        <v>0.005692863665587746</v>
       </c>
       <c r="D9" t="n">
-        <v>1.168571329360313</v>
+        <v>1.725873270857172</v>
       </c>
       <c r="E9" t="b">
         <v>0</v>
@@ -767,17 +802,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>OPCT_YN</t>
+          <t>LBST_EXE_CNT</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.5464846449371249</v>
+        <v>0.549257369890192</v>
       </c>
       <c r="C10" t="n">
-        <v>0.003663743761293497</v>
+        <v>0.003791115542932379</v>
       </c>
       <c r="D10" t="n">
-        <v>1.128880869382555</v>
+        <v>1.149331051405507</v>
       </c>
       <c r="E10" t="b">
         <v>0</v>
@@ -786,17 +821,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>LBST_EXE_CNT</t>
+          <t>TMNT_CLT_NUM</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.5444679008528904</v>
+        <v>0.546494090338714</v>
       </c>
       <c r="C11" t="n">
-        <v>0.00369384421156972</v>
+        <v>0.003728982782713846</v>
       </c>
       <c r="D11" t="n">
-        <v>1.138155487011554</v>
+        <v>1.1304946139981</v>
       </c>
       <c r="E11" t="b">
         <v>0</v>
@@ -805,17 +840,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CUMU_PYHWY_EXE_AMT</t>
+          <t>LBST_PLAN_RT</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.5435407363211828</v>
+        <v>0.5445845128778724</v>
       </c>
       <c r="C12" t="n">
-        <v>0.003560921462815187</v>
+        <v>0.00390130950783065</v>
       </c>
       <c r="D12" t="n">
-        <v>1.097199034281422</v>
+        <v>1.182737932335627</v>
       </c>
       <c r="E12" t="b">
         <v>0</v>
@@ -824,17 +859,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>LBST_PLAN_RT</t>
+          <t>CUMU_PYHWY_EXE_CNT</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.5420107215366481</v>
+        <v>0.5436159780519747</v>
       </c>
       <c r="C13" t="n">
-        <v>0.00380586140159499</v>
+        <v>0.003756337315938071</v>
       </c>
       <c r="D13" t="n">
-        <v>1.172670472529229</v>
+        <v>1.138787533080958</v>
       </c>
       <c r="E13" t="b">
         <v>0</v>
@@ -847,13 +882,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.5408115195586706</v>
+        <v>0.5428638312693133</v>
       </c>
       <c r="C14" t="n">
-        <v>0.003580103909639817</v>
+        <v>0.003615649289667215</v>
       </c>
       <c r="D14" t="n">
-        <v>1.103109572424686</v>
+        <v>1.096135940080715</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -862,17 +897,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>LAF_CD</t>
+          <t>TMNT_CORP_CLT_NUM</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.5396393502764638</v>
+        <v>0.5411646160592046</v>
       </c>
       <c r="C15" t="n">
-        <v>0.004214741324079186</v>
+        <v>0.003947984377281862</v>
       </c>
       <c r="D15" t="n">
-        <v>1.29865546286711</v>
+        <v>1.196888088450121</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -885,13 +920,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.5392026379213561</v>
+        <v>0.5399526557139638</v>
       </c>
       <c r="C16" t="n">
-        <v>0.003522438628760229</v>
+        <v>0.003632431637654578</v>
       </c>
       <c r="D16" t="n">
-        <v>1.085341617934999</v>
+        <v>1.101223749576083</v>
       </c>
       <c r="E16" t="b">
         <v>0</v>
@@ -900,17 +935,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>AID_BIZ_EXE_TY_CD</t>
+          <t>CUMU_PYHWY_EXE_AMT</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.5368930610192355</v>
+        <v>0.5397321452784584</v>
       </c>
       <c r="C17" t="n">
-        <v>0.003517556737091153</v>
+        <v>0.003596629212680411</v>
       </c>
       <c r="D17" t="n">
-        <v>1.083837398625275</v>
+        <v>1.090369730944248</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -919,17 +954,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>BIZ_MDCN</t>
+          <t>LBST_EXE_AVG_AMT</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.5362428540281104</v>
+        <v>0.5375056812269929</v>
       </c>
       <c r="C18" t="n">
-        <v>0.003583608447263103</v>
+        <v>0.003735201711269473</v>
       </c>
       <c r="D18" t="n">
-        <v>1.104189398345035</v>
+        <v>1.132379971385526</v>
       </c>
       <c r="E18" t="b">
         <v>0</v>
@@ -938,17 +973,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>LBST_EXE_AVG_AMT</t>
+          <t>TMNT_INDV_BZR_CLT_NUM</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.5339217389068401</v>
+        <v>0.5367795722044035</v>
       </c>
       <c r="C19" t="n">
-        <v>0.003611332294837258</v>
+        <v>0.00364203013711108</v>
       </c>
       <c r="D19" t="n">
-        <v>1.112731731868133</v>
+        <v>1.104133672354043</v>
       </c>
       <c r="E19" t="b">
         <v>0</v>
@@ -957,17 +992,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>LODI_CNT</t>
+          <t>ETC_EXE_CNT</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.5325959425035319</v>
+        <v>0.5362190782905764</v>
       </c>
       <c r="C20" t="n">
-        <v>0.003522441688832761</v>
+        <v>0.003673514521931621</v>
       </c>
       <c r="D20" t="n">
-        <v>1.085342560811348</v>
+        <v>1.113678615181256</v>
       </c>
       <c r="E20" t="b">
         <v>0</v>
@@ -976,17 +1011,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>TMNT_CLT_NUM</t>
+          <t>LODI_CNT</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0.5323037213752917</v>
+        <v>0.5347050272341033</v>
       </c>
       <c r="C21" t="n">
-        <v>0.003614848678399931</v>
+        <v>0.003602585244128015</v>
       </c>
       <c r="D21" t="n">
-        <v>1.11381520778565</v>
+        <v>1.092175387302742</v>
       </c>
       <c r="E21" t="b">
         <v>0</v>
@@ -995,17 +1030,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>AID_BIZ_DPI_DV_CD</t>
+          <t>LAF_CD</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>0.5292940530079201</v>
+        <v>0.5344274074045279</v>
       </c>
       <c r="C22" t="n">
-        <v>0.003447784372087854</v>
+        <v>0.00411741339066379</v>
       </c>
       <c r="D22" t="n">
-        <v>1.062338982470759</v>
+        <v>1.248252923914415</v>
       </c>
       <c r="E22" t="b">
         <v>0</v>
@@ -1014,17 +1049,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>LAF_CPRN_AID_BIZCT_RT</t>
+          <t>BIZ_MDCN</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>0.5283204087837603</v>
+        <v>0.5316615690560564</v>
       </c>
       <c r="C23" t="n">
-        <v>0.003597886647225243</v>
+        <v>0.003575825378118196</v>
       </c>
       <c r="D23" t="n">
-        <v>1.108588829046702</v>
+        <v>1.084062750115022</v>
       </c>
       <c r="E23" t="b">
         <v>0</v>
@@ -1033,17 +1068,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CUMU_SBAT_EXE_RTRCN_SUM_AMT</t>
+          <t>AID_BIZ_DPI_DV_CD</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>0.5276086138227275</v>
+        <v>0.5312885510365969</v>
       </c>
       <c r="C24" t="n">
-        <v>0.003595269992398425</v>
+        <v>0.003519091765955575</v>
       </c>
       <c r="D24" t="n">
-        <v>1.107782579546674</v>
+        <v>1.066863141878745</v>
       </c>
       <c r="E24" t="b">
         <v>0</v>
@@ -1052,17 +1087,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CUMU_SBAT_EXE_RTRCN_CNT</t>
+          <t>TMNT_CORP_DLNG_AMT</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>0.5273963230484093</v>
+        <v>0.5267355860777962</v>
       </c>
       <c r="C25" t="n">
-        <v>0.003508039652314369</v>
+        <v>0.003541232479017544</v>
       </c>
       <c r="D25" t="n">
-        <v>1.080904973314775</v>
+        <v>1.073575416599525</v>
       </c>
       <c r="E25" t="b">
         <v>0</v>
@@ -1071,17 +1106,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CONT_BIZ_YN</t>
+          <t>CORP_BZR_CUMU_EXE_CNT</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>0.5263770990173797</v>
+        <v>0.5262871650099309</v>
       </c>
       <c r="C26" t="n">
-        <v>0.003431180505697649</v>
+        <v>0.003538900491734144</v>
       </c>
       <c r="D26" t="n">
-        <v>1.057222962261128</v>
+        <v>1.072868441207733</v>
       </c>
       <c r="E26" t="b">
         <v>0</v>
@@ -1094,13 +1129,13 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>0.5261580526645433</v>
+        <v>0.5256072341678238</v>
       </c>
       <c r="C27" t="n">
-        <v>0.003480421910136889</v>
+        <v>0.003510008630121882</v>
       </c>
       <c r="D27" t="n">
-        <v>1.07239533322229</v>
+        <v>1.064109458974709</v>
       </c>
       <c r="E27" t="b">
         <v>0</v>
@@ -1109,17 +1144,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>PBAC_TY_DV_CD</t>
+          <t>SECT_CD</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>0.5258992581122339</v>
+        <v>0.5252018201778955</v>
       </c>
       <c r="C28" t="n">
-        <v>0.003423424015914176</v>
+        <v>0.003800308173116553</v>
       </c>
       <c r="D28" t="n">
-        <v>1.0548330153924</v>
+        <v>1.152117929092328</v>
       </c>
       <c r="E28" t="b">
         <v>0</v>
@@ -1132,13 +1167,13 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>0.5254248477353729</v>
+        <v>0.5250593577702061</v>
       </c>
       <c r="C29" t="n">
-        <v>0.003454149577878362</v>
+        <v>0.003510376875017002</v>
       </c>
       <c r="D29" t="n">
-        <v>1.064300243823832</v>
+        <v>1.064221097696265</v>
       </c>
       <c r="E29" t="b">
         <v>0</v>
@@ -1147,17 +1182,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>PRIV_AID_BIZ_CGP_YN</t>
+          <t>SBAT_BDTR_CRCD_EXE_CNT</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>0.5253439024666549</v>
+        <v>0.5250466200090056</v>
       </c>
       <c r="C30" t="n">
-        <v>0.003421221114454581</v>
+        <v>0.003613490121119549</v>
       </c>
       <c r="D30" t="n">
-        <v>1.054154252499333</v>
+        <v>1.095481357167336</v>
       </c>
       <c r="E30" t="b">
         <v>0</v>
@@ -1166,17 +1201,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>TMNT_INDV_BZR_CLT_NUM</t>
+          <t>CONT_BIZ_YN</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>0.5253388154346381</v>
+        <v>0.5248718769511289</v>
       </c>
       <c r="C31" t="n">
-        <v>0.003532912943437238</v>
+        <v>0.003475701110872133</v>
       </c>
       <c r="D31" t="n">
-        <v>1.088568987049534</v>
+        <v>1.053708642454111</v>
       </c>
       <c r="E31" t="b">
         <v>0</v>
@@ -1185,17 +1220,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>INST_TY_CD</t>
+          <t>TMNT_EXE_CNT</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>0.5233817578085069</v>
+        <v>0.5247734201062337</v>
       </c>
       <c r="C32" t="n">
-        <v>0.003482533176817451</v>
+        <v>0.003494915553477982</v>
       </c>
       <c r="D32" t="n">
-        <v>1.073045861403608</v>
+        <v>1.059533776315705</v>
       </c>
       <c r="E32" t="b">
         <v>0</v>
@@ -1204,17 +1239,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>FYR</t>
+          <t>INST_TY_CD</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>0.5211636087832021</v>
+        <v>0.5244998927102782</v>
       </c>
       <c r="C33" t="n">
-        <v>0.003493648674309353</v>
+        <v>0.003539452500957447</v>
       </c>
       <c r="D33" t="n">
-        <v>1.076470793191918</v>
+        <v>1.073035790721041</v>
       </c>
       <c r="E33" t="b">
         <v>0</v>
@@ -1223,17 +1258,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ETC_EXE_CNT</t>
+          <t>BIZCT_SUM_AMT</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>0.521159305777018</v>
+        <v>0.5242186117695593</v>
       </c>
       <c r="C34" t="n">
-        <v>0.003481338638157068</v>
+        <v>0.003738662492270207</v>
       </c>
       <c r="D34" t="n">
-        <v>1.072677797497041</v>
+        <v>1.133429156782598</v>
       </c>
       <c r="E34" t="b">
         <v>0</v>
@@ -1242,17 +1277,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>BIZCT_SUM_AMT</t>
+          <t>CORP_BZR_CUMU_EXE_AMT</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>0.5208445131762683</v>
+        <v>0.5239794018015742</v>
       </c>
       <c r="C35" t="n">
-        <v>0.003563029752492529</v>
+        <v>0.003563216986361382</v>
       </c>
       <c r="D35" t="n">
-        <v>1.097848645181892</v>
+        <v>1.080240335316453</v>
       </c>
       <c r="E35" t="b">
         <v>0</v>
@@ -1261,17 +1296,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ODN_CAPT_DV_CD</t>
+          <t>PRIV_AID_BIZ_CGP_YN</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>0.5202024678608377</v>
+        <v>0.5232060332143686</v>
       </c>
       <c r="C36" t="n">
-        <v>0.003381870465804889</v>
+        <v>0.003461165180058938</v>
       </c>
       <c r="D36" t="n">
-        <v>1.042029443191504</v>
+        <v>1.049301866544621</v>
       </c>
       <c r="E36" t="b">
         <v>0</v>
@@ -1280,17 +1315,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>THY_PFM_AID_BIZ_NUM</t>
+          <t>TMNT_EXE_AMT</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>0.5200161728582947</v>
+        <v>0.5228311905900279</v>
       </c>
       <c r="C37" t="n">
-        <v>0.003324221225866052</v>
+        <v>0.003590374328599662</v>
       </c>
       <c r="D37" t="n">
-        <v>1.024266431272127</v>
+        <v>1.088473473123684</v>
       </c>
       <c r="E37" t="b">
         <v>0</v>
@@ -1299,17 +1334,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ACNT_DV_CD</t>
+          <t>INDV_CUMU_EXE_CNT</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>0.5196067552330154</v>
+        <v>0.5225820716960751</v>
       </c>
       <c r="C38" t="n">
-        <v>0.003564583272714486</v>
+        <v>0.003513001674533521</v>
       </c>
       <c r="D38" t="n">
-        <v>1.098327319284949</v>
+        <v>1.065016843316225</v>
       </c>
       <c r="E38" t="b">
         <v>0</v>
@@ -1318,17 +1353,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>AID_BIZ_DV_CD</t>
+          <t>INDV_BZR_CUMU_EXE_AMT</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>0.5192295698731296</v>
+        <v>0.5223263147040678</v>
       </c>
       <c r="C39" t="n">
-        <v>0.003379612163459114</v>
+        <v>0.0034818484595543</v>
       </c>
       <c r="D39" t="n">
-        <v>1.041333610054274</v>
+        <v>1.055572299376254</v>
       </c>
       <c r="E39" t="b">
         <v>0</v>
@@ -1337,17 +1372,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CARD_FR_USE_CNT</t>
+          <t>INDV_BZR_CUMU_EXE_CNT</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>0.5170874609718751</v>
+        <v>0.5221836487417177</v>
       </c>
       <c r="C40" t="n">
-        <v>0.003378631456029198</v>
+        <v>0.003460881981067638</v>
       </c>
       <c r="D40" t="n">
-        <v>1.041031432301619</v>
+        <v>1.04921601070859</v>
       </c>
       <c r="E40" t="b">
         <v>0</v>
@@ -1356,17 +1391,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>LAF_PFM_AID_BIZ_NUM</t>
+          <t>PBAC_TY_DV_CD</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>0.5169179855658851</v>
+        <v>0.5221449446287328</v>
       </c>
       <c r="C41" t="n">
-        <v>0.003367512876676662</v>
+        <v>0.003451246101084407</v>
       </c>
       <c r="D41" t="n">
-        <v>1.037605550923561</v>
+        <v>1.046294755487817</v>
       </c>
       <c r="E41" t="b">
         <v>0</v>
@@ -1375,17 +1410,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>TMNT_EXE_AMT</t>
+          <t>AID_BIZ_DV_CD</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>0.516696102517889</v>
+        <v>0.5214768728975676</v>
       </c>
       <c r="C42" t="n">
-        <v>0.003565527458554109</v>
+        <v>0.003450561736219478</v>
       </c>
       <c r="D42" t="n">
-        <v>1.098618243924044</v>
+        <v>1.046087280463422</v>
       </c>
       <c r="E42" t="b">
         <v>0</v>
@@ -1394,17 +1429,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>INDV_BZR_CUMU_EXE_AMT</t>
+          <t>ODN_CAPT_DV_CD</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>0.5163873624470696</v>
+        <v>0.5211339050452704</v>
       </c>
       <c r="C43" t="n">
-        <v>0.003440438999690085</v>
+        <v>0.003443838891536111</v>
       </c>
       <c r="D43" t="n">
-        <v>1.060075710004508</v>
+        <v>1.044049153674389</v>
       </c>
       <c r="E43" t="b">
         <v>0</v>
@@ -1413,17 +1448,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CARD_RTRCN_CNT</t>
+          <t>LAF_CPRN_AID_BIZCT_RT</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>0.5159450497887964</v>
+        <v>0.5207652979239803</v>
       </c>
       <c r="C44" t="n">
-        <v>0.003370333263437088</v>
+        <v>0.003585919085862689</v>
       </c>
       <c r="D44" t="n">
-        <v>1.03847457475971</v>
+        <v>1.087122802388075</v>
       </c>
       <c r="E44" t="b">
         <v>0</v>
@@ -1432,17 +1467,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>EXE_PLAN_CHG_TMS</t>
+          <t>TMNT_INDV_BZR_DLNG_AMT</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>0.5158741398846266</v>
+        <v>0.5203631522996103</v>
       </c>
       <c r="C45" t="n">
-        <v>0.003355703063720464</v>
+        <v>0.00362609780539213</v>
       </c>
       <c r="D45" t="n">
-        <v>1.033966685111469</v>
+        <v>1.099303557481913</v>
       </c>
       <c r="E45" t="b">
         <v>0</v>
@@ -1451,17 +1486,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>TMNT_CORP_CLT_NUM</t>
+          <t>INDV_CUMU_EXE_AMT</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>0.5158158233953907</v>
+        <v>0.52036040061816</v>
       </c>
       <c r="C46" t="n">
-        <v>0.003571445535361535</v>
+        <v>0.003533804053500495</v>
       </c>
       <c r="D46" t="n">
-        <v>1.10044173490123</v>
+        <v>1.071323382860877</v>
       </c>
       <c r="E46" t="b">
         <v>0</v>
@@ -1470,17 +1505,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>LBST_EXE_RT_DV_CD</t>
+          <t>TMNT_INDV_DLNG_AMT</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>0.5149116792408132</v>
+        <v>0.5195868666427925</v>
       </c>
       <c r="C47" t="n">
-        <v>0.003413090430529153</v>
+        <v>0.003393201899416258</v>
       </c>
       <c r="D47" t="n">
-        <v>1.051649008100044</v>
+        <v>1.02869782324564</v>
       </c>
       <c r="E47" t="b">
         <v>0</v>
@@ -1489,17 +1524,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>TMNT_EXE_CNT</t>
+          <t>AID_BIZ_EXE_TY_CD</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>0.514261549904789</v>
+        <v>0.5184749172986963</v>
       </c>
       <c r="C48" t="n">
-        <v>0.003355144383326447</v>
+        <v>0.003427304778271853</v>
       </c>
       <c r="D48" t="n">
-        <v>1.033794543266952</v>
+        <v>1.039036600095669</v>
       </c>
       <c r="E48" t="b">
         <v>0</v>
@@ -1508,17 +1543,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>INDV_CUMU_EXE_CNT</t>
+          <t>LAF_PFM_AID_BIZ_NUM</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>0.5115497224864157</v>
+        <v>0.5181296491966558</v>
       </c>
       <c r="C49" t="n">
-        <v>0.003381430773260546</v>
+        <v>0.003430482669280371</v>
       </c>
       <c r="D49" t="n">
-        <v>1.041893964147647</v>
+        <v>1.040000023334215</v>
       </c>
       <c r="E49" t="b">
         <v>0</v>
@@ -1527,17 +1562,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>RPRSV_HSHD_DV_CD</t>
+          <t>ACNT_DV_CD</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>0.5110866082275073</v>
+        <v>0.5172478618979596</v>
       </c>
       <c r="C50" t="n">
-        <v>0.01582347427300902</v>
+        <v>0.003553241500796928</v>
       </c>
       <c r="D50" t="n">
-        <v>4.875564056275702</v>
+        <v>1.077216123792895</v>
       </c>
       <c r="E50" t="b">
         <v>0</v>
@@ -1546,17 +1581,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>TMNT_INDV_BZR_DLNG_AMT</t>
+          <t>CUMU_SBAT_EXE_RTRCN_CNT</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>0.5103821527116879</v>
+        <v>0.5167220752849407</v>
       </c>
       <c r="C51" t="n">
-        <v>0.003446195810906694</v>
+        <v>0.003529509827033251</v>
       </c>
       <c r="D51" t="n">
-        <v>1.061849511469484</v>
+        <v>1.070021526516833</v>
       </c>
       <c r="E51" t="b">
         <v>0</v>
@@ -1565,17 +1600,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>INDV_CUMU_EXE_AMT</t>
+          <t>CUMU_SBAT_EXE_RTRCN_SUM_AMT</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>0.5100964982150622</v>
+        <v>0.5166966239756949</v>
       </c>
       <c r="C52" t="n">
-        <v>0.003460614357021484</v>
+        <v>0.00352439984533589</v>
       </c>
       <c r="D52" t="n">
-        <v>1.066292185939586</v>
+        <v>1.068472362274703</v>
       </c>
       <c r="E52" t="b">
         <v>0</v>
@@ -1584,17 +1619,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>TMNT_SBAT_EXE_RTRCN_CNT</t>
+          <t>EXE_PLAN_CHG_TMS</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>0.5097223380819718</v>
+        <v>0.5158356021251265</v>
       </c>
       <c r="C53" t="n">
-        <v>0.003340206920701427</v>
+        <v>0.003409795449209062</v>
       </c>
       <c r="D53" t="n">
-        <v>1.02919197908857</v>
+        <v>1.033728395860465</v>
       </c>
       <c r="E53" t="b">
         <v>0</v>
@@ -1603,17 +1638,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>TMNT_SBAT_EXE_RTRCN_SUM_AMT</t>
+          <t>FYR</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>0.5097172996363016</v>
+        <v>0.5154195072610115</v>
       </c>
       <c r="C54" t="n">
-        <v>0.003368872853955759</v>
+        <v>0.003507990513204805</v>
       </c>
       <c r="D54" t="n">
-        <v>1.038024590144968</v>
+        <v>1.063497637886194</v>
       </c>
       <c r="E54" t="b">
         <v>0</v>
@@ -1622,17 +1657,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>BIZCT_SBAT_AMT</t>
+          <t>CARD_FR_USE_CNT</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>0.5096960200622909</v>
+        <v>0.5145462639229582</v>
       </c>
       <c r="C55" t="n">
-        <v>0.003437294063891046</v>
+        <v>0.00341192188332316</v>
       </c>
       <c r="D55" t="n">
-        <v>1.059106685397362</v>
+        <v>1.03437305486081</v>
       </c>
       <c r="E55" t="b">
         <v>0</v>
@@ -1641,17 +1676,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>SBAT_BDTR_CEK_CARD_EXE_CNT</t>
+          <t>CARD_RTRCN_CNT</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>0.5088206448386565</v>
+        <v>0.5141839169282661</v>
       </c>
       <c r="C56" t="n">
-        <v>0.003483479100347937</v>
+        <v>0.00343765556717192</v>
       </c>
       <c r="D56" t="n">
-        <v>1.073337321463874</v>
+        <v>1.042174590208254</v>
       </c>
       <c r="E56" t="b">
         <v>0</v>
@@ -1660,17 +1695,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>INDV_BZR_CUMU_EXE_CNT</t>
+          <t>LBST_EXE_RT_DV_CD</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>0.5087932774369425</v>
+        <v>0.5141152681189816</v>
       </c>
       <c r="C57" t="n">
-        <v>0.003324219592079169</v>
+        <v>0.003456164864275467</v>
       </c>
       <c r="D57" t="n">
-        <v>1.024265927866083</v>
+        <v>1.047785949097185</v>
       </c>
       <c r="E57" t="b">
         <v>0</v>
@@ -1679,17 +1714,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>INVC_EXE_CNT</t>
+          <t>BIZCT_SBAT_AMT</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>0.5073025943381575</v>
+        <v>0.5139523525718271</v>
       </c>
       <c r="C58" t="n">
-        <v>0.003300668094053085</v>
+        <v>0.003616307592596751</v>
       </c>
       <c r="D58" t="n">
-        <v>1.017009187957623</v>
+        <v>1.096335514055599</v>
       </c>
       <c r="E58" t="b">
         <v>0</v>
@@ -1702,13 +1737,13 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>0.5071974293985568</v>
+        <v>0.5137048243590526</v>
       </c>
       <c r="C59" t="n">
-        <v>0.003380306708912013</v>
+        <v>0.003328432872420129</v>
       </c>
       <c r="D59" t="n">
-        <v>1.041547614942656</v>
+        <v>1.009062163753607</v>
       </c>
       <c r="E59" t="b">
         <v>0</v>
@@ -1717,17 +1752,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>PRIV_AID_BZR_YN</t>
+          <t>FLD_CD</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>0.5065540813876619</v>
+        <v>0.5134020384429917</v>
       </c>
       <c r="C60" t="n">
-        <v>0.003288455027911747</v>
+        <v>0.00366600489520257</v>
       </c>
       <c r="D60" t="n">
-        <v>1.013246070878007</v>
+        <v>1.11140196413055</v>
       </c>
       <c r="E60" t="b">
         <v>0</v>
@@ -1736,17 +1771,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>TMNT_INDV_DLNG_AMT</t>
+          <t>SBAT_BDTR_CEK_CARD_EXE_CNT</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>0.5062834035285614</v>
+        <v>0.5123333600591847</v>
       </c>
       <c r="C61" t="n">
-        <v>0.003287188609086437</v>
+        <v>0.003511554944411213</v>
       </c>
       <c r="D61" t="n">
-        <v>1.012855859095289</v>
+        <v>1.064578246329733</v>
       </c>
       <c r="E61" t="b">
         <v>0</v>
@@ -1755,17 +1790,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>FLD_CD</t>
+          <t>DEPT_CD</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>0.5058392429280455</v>
+        <v>0.5122030809724812</v>
       </c>
       <c r="C62" t="n">
-        <v>0.003350829880802737</v>
+        <v>0.00324356746140329</v>
       </c>
       <c r="D62" t="n">
-        <v>1.032465149161563</v>
+        <v>0.9833339972107065</v>
       </c>
       <c r="E62" t="b">
         <v>0</v>
@@ -1774,17 +1809,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>SBAT_BDTR_CRCD_EXE_CNT</t>
+          <t>ETI_EXE_CNT</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>0.505462729056386</v>
+        <v>0.5111914537070147</v>
       </c>
       <c r="C63" t="n">
-        <v>0.003385789540039949</v>
+        <v>0.00342028045020009</v>
       </c>
       <c r="D63" t="n">
-        <v>1.043236997053865</v>
+        <v>1.036907074293379</v>
       </c>
       <c r="E63" t="b">
         <v>0</v>
@@ -1793,17 +1828,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>PRTC_MNPW_N_LBST_GIVE_AVG_AMT</t>
+          <t>PRIV_AID_BZR_YN</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>0.5050176486374277</v>
+        <v>0.5108458215868614</v>
       </c>
       <c r="C64" t="n">
-        <v>0.003311418286362922</v>
+        <v>0.003371485541423886</v>
       </c>
       <c r="D64" t="n">
-        <v>1.020321561101446</v>
+        <v>1.022114197850576</v>
       </c>
       <c r="E64" t="b">
         <v>0</v>
@@ -1812,17 +1847,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>PRTC_MNPW_N_LBST_GIVE_CNT</t>
+          <t>THY_PFM_AID_BIZ_NUM</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>0.5049399835700077</v>
+        <v>0.5096798481792161</v>
       </c>
       <c r="C65" t="n">
-        <v>0.003255388777023212</v>
+        <v>0.003309172958254548</v>
       </c>
       <c r="D65" t="n">
-        <v>1.003057624173674</v>
+        <v>1.003223244536498</v>
       </c>
       <c r="E65" t="b">
         <v>0</v>
@@ -1831,17 +1866,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>PRTC_MNPW_N_LBST_GIVE_AMT</t>
+          <t>TMNT_DLNG_AMT</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>0.5047469226072485</v>
+        <v>0.5080576463975297</v>
       </c>
       <c r="C66" t="n">
-        <v>0.003233363701681251</v>
+        <v>0.003462298007492507</v>
       </c>
       <c r="D66" t="n">
-        <v>0.9962712090146975</v>
+        <v>1.049645299428831</v>
       </c>
       <c r="E66" t="b">
         <v>0</v>
@@ -1850,17 +1885,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>ETI_EXE_CNT</t>
+          <t>SBAT_EXE_SUM_AMT</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>0.5043638520704046</v>
+        <v>0.5080572093295588</v>
       </c>
       <c r="C67" t="n">
-        <v>0.003293738443247539</v>
+        <v>0.003462293137727503</v>
       </c>
       <c r="D67" t="n">
-        <v>1.014874008552195</v>
+        <v>1.049643823089725</v>
       </c>
       <c r="E67" t="b">
         <v>0</v>
@@ -1869,17 +1904,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CUMU_EXE_AMT</t>
+          <t>TMNT_SBAT_EXE_RTRCN_CNT</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>0.5042593457457246</v>
+        <v>0.5079414741412761</v>
       </c>
       <c r="C68" t="n">
-        <v>0.003309959930171629</v>
+        <v>0.003383854859123062</v>
       </c>
       <c r="D68" t="n">
-        <v>1.019872209150994</v>
+        <v>1.025864133919622</v>
       </c>
       <c r="E68" t="b">
         <v>0</v>
@@ -1888,17 +1923,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>EVENT_FSTV_YN</t>
+          <t>TMNT_SBAT_EXE_RTRCN_SUM_AMT</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>0.5042373282406204</v>
+        <v>0.507843981718664</v>
       </c>
       <c r="C69" t="n">
-        <v>0.003283236679381769</v>
+        <v>0.00336021106630494</v>
       </c>
       <c r="D69" t="n">
-        <v>1.011638181732621</v>
+        <v>1.018696179012648</v>
       </c>
       <c r="E69" t="b">
         <v>0</v>
@@ -1907,17 +1942,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CORP_BZR_CUMU_EXE_CNT</t>
+          <t>PBCN_DGR</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>0.5040854768051439</v>
+        <v>0.5063179000072006</v>
       </c>
       <c r="C70" t="n">
-        <v>0.003301821808960061</v>
+        <v>0.003340617298244728</v>
       </c>
       <c r="D70" t="n">
-        <v>1.017364673158571</v>
+        <v>1.012756047199039</v>
       </c>
       <c r="E70" t="b">
         <v>0</v>
@@ -1926,17 +1961,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>NTN_DRCT_BIZ_YN</t>
+          <t>VNCL_GOEM_VRSC_YN</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>0.5040737591902528</v>
+        <v>0.5036531281892829</v>
       </c>
       <c r="C71" t="n">
-        <v>0.003292080288896853</v>
+        <v>0.003322739254964285</v>
       </c>
       <c r="D71" t="n">
-        <v>1.014363094348874</v>
+        <v>1.007336061960423</v>
       </c>
       <c r="E71" t="b">
         <v>0</v>
@@ -1945,17 +1980,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>SECT_CD</t>
+          <t>EVENT_FSTV_YN</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>0.5035697165404435</v>
+        <v>0.5032134796706612</v>
       </c>
       <c r="C72" t="n">
-        <v>0.003460520950933457</v>
+        <v>0.003325691938189675</v>
       </c>
       <c r="D72" t="n">
-        <v>1.066263405448175</v>
+        <v>1.008231210229441</v>
       </c>
       <c r="E72" t="b">
         <v>0</v>
@@ -1968,13 +2003,13 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>0.503129107726445</v>
+        <v>0.5028787520885858</v>
       </c>
       <c r="C73" t="n">
-        <v>0.003265837539623402</v>
+        <v>0.003317579142632282</v>
       </c>
       <c r="D73" t="n">
-        <v>1.006277120125517</v>
+        <v>1.005771699897396</v>
       </c>
       <c r="E73" t="b">
         <v>0</v>
@@ -1983,17 +2018,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CORP_BZR_CUMU_EXE_AMT</t>
+          <t>LTST_Y1_WTHN_OPBIZ_CLT_CNT</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>0.5031060898409222</v>
+        <v>0.5026470395804683</v>
       </c>
       <c r="C74" t="n">
-        <v>0.003332726814101617</v>
+        <v>0.00331471214409166</v>
       </c>
       <c r="D74" t="n">
-        <v>1.026887192020577</v>
+        <v>1.004902528169509</v>
       </c>
       <c r="E74" t="b">
         <v>0</v>
@@ -2002,17 +2037,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>VNCL_GOEM_VRSC_YN</t>
+          <t>INVC_EXE_CNT</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>0.5027770286344506</v>
+        <v>0.5026115110843458</v>
       </c>
       <c r="C75" t="n">
-        <v>0.003263533460838379</v>
+        <v>0.003315810374828015</v>
       </c>
       <c r="D75" t="n">
-        <v>1.005567182250101</v>
+        <v>1.005235472568752</v>
       </c>
       <c r="E75" t="b">
         <v>0</v>
@@ -2021,17 +2056,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>LTST_Y1_WTHN_OPBIZ_CLT_CNT</t>
+          <t>RPRSV_HSHD_DV_CD</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>0.5019247576720666</v>
+        <v>0.5024915332588026</v>
       </c>
       <c r="C76" t="n">
-        <v>0.003258027815122984</v>
+        <v>0.01795364480224983</v>
       </c>
       <c r="D76" t="n">
-        <v>1.003870770457505</v>
+        <v>5.442904924277287</v>
       </c>
       <c r="E76" t="b">
         <v>0</v>
@@ -2040,17 +2075,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>LSA_MNG_CMMT_DLBR_YN</t>
+          <t>NTN_DRCT_BIZ_YN</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>0.5018066048130083</v>
+        <v>0.502398116033327</v>
       </c>
       <c r="C77" t="n">
-        <v>0.003264822394257026</v>
+        <v>0.003321382007854289</v>
       </c>
       <c r="D77" t="n">
-        <v>1.005964331279351</v>
+        <v>1.006924593032535</v>
       </c>
       <c r="E77" t="b">
         <v>0</v>
@@ -2059,17 +2094,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>TMNT_DLNG_AMT</t>
+          <t>LSA_MNG_CMMT_DLBR_YN</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>0.501789880728077</v>
+        <v>0.5022441737173295</v>
       </c>
       <c r="C78" t="n">
-        <v>0.003326103108533695</v>
+        <v>0.003325328633408133</v>
       </c>
       <c r="D78" t="n">
-        <v>1.024846281141643</v>
+        <v>1.008121069174171</v>
       </c>
       <c r="E78" t="b">
         <v>0</v>
@@ -2078,17 +2113,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>SBAT_EXE_SUM_AMT</t>
+          <t>PRTC_MNPW_N_LBST_GIVE_AVG_AMT</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>0.5017894189501502</v>
+        <v>0.5021873396966008</v>
       </c>
       <c r="C79" t="n">
-        <v>0.003326097916930697</v>
+        <v>0.0033676944970224</v>
       </c>
       <c r="D79" t="n">
-        <v>1.024844681493391</v>
+        <v>1.02096488836672</v>
       </c>
       <c r="E79" t="b">
         <v>0</v>
@@ -2097,17 +2132,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>PBCN_DGR</t>
+          <t>PRTC_MNPW_N_LBST_GIVE_CNT</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>0.5012132085496424</v>
+        <v>0.5018453042559747</v>
       </c>
       <c r="C80" t="n">
-        <v>0.003253334018405725</v>
+        <v>0.003272532201537704</v>
       </c>
       <c r="D80" t="n">
-        <v>1.002424507382324</v>
+        <v>0.9921150736129897</v>
       </c>
       <c r="E80" t="b">
         <v>0</v>
@@ -2116,17 +2151,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>AST_LAT_RT</t>
+          <t>PRTC_MNPW_N_LBST_GIVE_AMT</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>0.5008661006299149</v>
+        <v>0.5018311658253051</v>
       </c>
       <c r="C81" t="n">
-        <v>0.003250909419827864</v>
+        <v>0.003276667216109198</v>
       </c>
       <c r="D81" t="n">
-        <v>1.001677434680516</v>
+        <v>0.9933686625873202</v>
       </c>
       <c r="E81" t="b">
         <v>0</v>
@@ -2135,17 +2170,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>DEPT_CD</t>
+          <t>RERE_DSCRD_CNT</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>0.5008418452459913</v>
+        <v>0.5009437787214805</v>
       </c>
       <c r="C82" t="n">
-        <v>0.003115840495814372</v>
+        <v>0.003529829313621818</v>
       </c>
       <c r="D82" t="n">
-        <v>0.9600596976603148</v>
+        <v>1.070118383458434</v>
       </c>
       <c r="E82" t="b">
         <v>0</v>
@@ -2154,17 +2189,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>TMNT_CORP_DLNG_AMT</t>
+          <t>CUMU_EXE_AMT</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>0.5003170213436747</v>
+        <v>0.5002495149226776</v>
       </c>
       <c r="C83" t="n">
-        <v>0.003231417296628579</v>
+        <v>0.003272426984630141</v>
       </c>
       <c r="D83" t="n">
-        <v>0.9956714783645235</v>
+        <v>0.9920831755983748</v>
       </c>
       <c r="E83" t="b">
         <v>0</v>
@@ -2173,17 +2208,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>RERE_DSCRD_CNT</t>
+          <t>AST_LAT_RT</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>0.500194525612712</v>
+        <v>0.5002031024081002</v>
       </c>
       <c r="C84" t="n">
-        <v>0.003323987596027563</v>
+        <v>0.003288177943345881</v>
       </c>
       <c r="D84" t="n">
-        <v>1.024194444727115</v>
+        <v>0.9968583046432163</v>
       </c>
       <c r="E84" t="b">
         <v>0</v>
@@ -2278,13 +2313,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.9999082090604214</v>
+        <v>0.9999227931151171</v>
       </c>
       <c r="C2" t="n">
         <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>1924</v>
+        <v>1961</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -2299,13 +2334,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.9968577994433535</v>
+        <v>0.9967901648284857</v>
       </c>
       <c r="C3" t="n">
         <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>63</v>
+        <v>54</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -2320,7 +2355,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.9967545346363276</v>
+        <v>0.9967014590458543</v>
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="n">
@@ -2343,6 +2378,261 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:U3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>그룹키(group_key)</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>전체행수(n_rows)</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Train행수(n_rows_train)</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Test행수(n_rows_test)</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>엔티티수(n_entities)</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Train엔티티수(n_entities_train)</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Test엔티티수(n_entities_test)</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>엔티티당평균행수(rows_per_entity_mean)</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>엔티티당최대행수(rows_per_entity_max)</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>양성행수(n_pos_rows)</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Test양성행수(n_pos_rows_test)</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>양성엔티티수(n_pos_entities)</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Train양성엔티티수(n_pos_entities_train)</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Test양성엔티티수(n_pos_entities_test)</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>양성엔티티당양성행수(pos_rows_per_pos_entity)</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>라벨고착성(label_stickiness)</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Test엔티티_Train중복비율(entity_overlap_ratio)</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Test양성엔티티_Train등장비율(pos_entity_seen_ratio)</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>Test양성엔티티_Train에서이미양성비율(pos_entity_seen_positive_ratio)</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>Test양성행_이미양성엔티티비율(pos_row_seen_positive_ratio)</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>랜덤분할기대중복비율(expected_overlap_under_random)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>PFM_BIZ_ID</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>871546</v>
+      </c>
+      <c r="C2" t="n">
+        <v>608754</v>
+      </c>
+      <c r="D2" t="n">
+        <v>262792</v>
+      </c>
+      <c r="E2" t="n">
+        <v>235378</v>
+      </c>
+      <c r="F2" t="n">
+        <v>164766</v>
+      </c>
+      <c r="G2" t="n">
+        <v>70614</v>
+      </c>
+      <c r="H2" t="n">
+        <v>3.702750469457639</v>
+      </c>
+      <c r="I2" t="n">
+        <v>24</v>
+      </c>
+      <c r="J2" t="n">
+        <v>2829</v>
+      </c>
+      <c r="K2" t="n">
+        <v>821</v>
+      </c>
+      <c r="L2" t="n">
+        <v>729</v>
+      </c>
+      <c r="M2" t="n">
+        <v>510</v>
+      </c>
+      <c r="N2" t="n">
+        <v>219</v>
+      </c>
+      <c r="O2" t="n">
+        <v>3.880658436213992</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0.8864929042912582</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>2.832299543999774e-05</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U2" t="n">
+        <v>0.894129845232883</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>PFM_BIZ_ID+INST_ID</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>871546</v>
+      </c>
+      <c r="C3" t="n">
+        <v>608754</v>
+      </c>
+      <c r="D3" t="n">
+        <v>262792</v>
+      </c>
+      <c r="E3" t="n">
+        <v>235380</v>
+      </c>
+      <c r="F3" t="n">
+        <v>164766</v>
+      </c>
+      <c r="G3" t="n">
+        <v>70614</v>
+      </c>
+      <c r="H3" t="n">
+        <v>3.70271900756224</v>
+      </c>
+      <c r="I3" t="n">
+        <v>24</v>
+      </c>
+      <c r="J3" t="n">
+        <v>2829</v>
+      </c>
+      <c r="K3" t="n">
+        <v>821</v>
+      </c>
+      <c r="L3" t="n">
+        <v>729</v>
+      </c>
+      <c r="M3" t="n">
+        <v>510</v>
+      </c>
+      <c r="N3" t="n">
+        <v>219</v>
+      </c>
+      <c r="O3" t="n">
+        <v>3.880658436213992</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0.8864929042912582</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S3" t="n">
+        <v>0</v>
+      </c>
+      <c r="T3" t="n">
+        <v>0</v>
+      </c>
+      <c r="U3" t="n">
+        <v>0.894129845232883</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:A84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>